<commit_message>
a few bug fixes and some additional docstrings
</commit_message>
<xml_diff>
--- a/compare/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
+++ b/compare/compare/subtract_out/files/subtract-out-csv-crosswalks.xlsx
@@ -9486,6 +9486,8 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
   <cols>
+    <col customWidth="1" min="2" max="2" width="26.0"/>
+    <col customWidth="1" min="4" max="4" width="31.63"/>
     <col customWidth="1" min="6" max="6" width="37.63"/>
   </cols>
   <sheetData>
@@ -11513,8 +11515,8 @@
     </row>
     <row r="103">
       <c r="A103" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B103" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11535,8 +11537,8 @@
     </row>
     <row r="104">
       <c r="A104" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B104" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11557,8 +11559,8 @@
     </row>
     <row r="105">
       <c r="A105" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B105" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11579,8 +11581,8 @@
     </row>
     <row r="106">
       <c r="A106" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B106" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11601,8 +11603,8 @@
     </row>
     <row r="107">
       <c r="A107" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B107" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11623,8 +11625,8 @@
     </row>
     <row r="108">
       <c r="A108" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B108" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-feedlot")</f>
@@ -11645,8 +11647,8 @@
     </row>
     <row r="109">
       <c r="A109" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B109" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11667,8 +11669,8 @@
     </row>
     <row r="110">
       <c r="A110" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B110" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11689,8 +11691,8 @@
     </row>
     <row r="111">
       <c r="A111" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B111" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11711,8 +11713,8 @@
     </row>
     <row r="112">
       <c r="A112" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B112" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11733,8 +11735,8 @@
     </row>
     <row r="113">
       <c r="A113" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B113" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11755,8 +11757,8 @@
     </row>
     <row r="114">
       <c r="A114" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B114" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-left-on-pasture-cattle")</f>
@@ -11777,8 +11779,8 @@
     </row>
     <row r="115">
       <c r="A115" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B115" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11799,8 +11801,8 @@
     </row>
     <row r="116">
       <c r="A116" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B116" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11821,8 +11823,8 @@
     </row>
     <row r="117">
       <c r="A117" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B117" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11843,8 +11845,8 @@
     </row>
     <row r="118">
       <c r="A118" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B118" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11865,8 +11867,8 @@
     </row>
     <row r="119">
       <c r="A119" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B119" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11887,8 +11889,8 @@
     </row>
     <row r="120">
       <c r="A120" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B120" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-cattle-feedlot")</f>
@@ -11909,8 +11911,8 @@
     </row>
     <row r="121">
       <c r="A121" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B121" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -11931,8 +11933,8 @@
     </row>
     <row r="122">
       <c r="A122" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B122" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -11953,8 +11955,8 @@
     </row>
     <row r="123">
       <c r="A123" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B123" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -11975,8 +11977,8 @@
     </row>
     <row r="124">
       <c r="A124" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B124" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -11997,8 +11999,8 @@
     </row>
     <row r="125">
       <c r="A125" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B125" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -12019,8 +12021,8 @@
     </row>
     <row r="126">
       <c r="A126" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B126" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-other")</f>
@@ -12041,8 +12043,8 @@
     </row>
     <row r="127">
       <c r="A127" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B127" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12063,8 +12065,8 @@
     </row>
     <row r="128">
       <c r="A128" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B128" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12085,8 +12087,8 @@
     </row>
     <row r="129">
       <c r="A129" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B129" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12107,8 +12109,8 @@
     </row>
     <row r="130">
       <c r="A130" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B130" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12129,8 +12131,8 @@
     </row>
     <row r="131">
       <c r="A131" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B131" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12151,8 +12153,8 @@
     </row>
     <row r="132">
       <c r="A132" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B132" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"manure-management-other")</f>
@@ -12173,8 +12175,8 @@
     </row>
     <row r="133">
       <c r="A133" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B133" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12195,8 +12197,8 @@
     </row>
     <row r="134">
       <c r="A134" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B134" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12217,8 +12219,8 @@
     </row>
     <row r="135">
       <c r="A135" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B135" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12239,8 +12241,8 @@
     </row>
     <row r="136">
       <c r="A136" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B136" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12261,8 +12263,8 @@
     </row>
     <row r="137">
       <c r="A137" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B137" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12283,8 +12285,8 @@
     </row>
     <row r="138">
       <c r="A138" s="9" t="b">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),TRUE)</f>
-        <v>1</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),FALSE)</f>
+        <v>0</v>
       </c>
       <c r="B138" s="9" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"enteric-fermentation-cattle-pasture")</f>
@@ -12820,6 +12822,10 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="3" max="3" width="14.38"/>
+    <col customWidth="1" min="4" max="4" width="32.63"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="str">
@@ -12879,8 +12885,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D3" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii Heat Plants")</f>
-        <v>1.A.1.a.iii Heat Plants</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iii  Heat Plants")</f>
+        <v>1.A.1.a.iii  Heat Plants</v>
       </c>
       <c r="E3" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -12901,8 +12907,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D4" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iv Other")</f>
-        <v>1.A.1.a.iv Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.1.a.iv  Other")</f>
+        <v>1.A.1.a.iv  Other</v>
       </c>
       <c r="E4" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -12945,8 +12951,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D6" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.b Road Transportation")</f>
-        <v>1.A.3.b Road Transportation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.b  Road Transportation")</f>
+        <v>1.A.3.b  Road Transportation</v>
       </c>
       <c r="E6" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -12967,8 +12973,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D7" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.c Railways")</f>
-        <v>1.A.3.c Railways</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.c  Railways")</f>
+        <v>1.A.3.c  Railways</v>
       </c>
       <c r="E7" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -12989,8 +12995,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D8" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.d Domestic Navigation")</f>
-        <v>1.A.3.d Domestic Navigation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.d  Domestic Navigation")</f>
+        <v>1.A.3.d  Domestic Navigation</v>
       </c>
       <c r="E8" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13011,8 +13017,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D9" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.e Other Transportation")</f>
-        <v>1.A.3.e Other Transportation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.e  Other Transportation")</f>
+        <v>1.A.3.e  Other Transportation</v>
       </c>
       <c r="E9" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13081,8 +13087,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D13" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.a Domestic Aviation")</f>
-        <v>1.A.3.a Domestic Aviation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.a  Domestic Aviation")</f>
+        <v>1.A.3.a  Domestic Aviation</v>
       </c>
       <c r="E13" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13103,8 +13109,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D14" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.b Road Transportation")</f>
-        <v>1.A.3.b Road Transportation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.b  Road Transportation")</f>
+        <v>1.A.3.b  Road Transportation</v>
       </c>
       <c r="E14" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13125,8 +13131,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D15" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.c Railways")</f>
-        <v>1.A.3.c Railways</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.c  Railways")</f>
+        <v>1.A.3.c  Railways</v>
       </c>
       <c r="E15" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13147,8 +13153,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D16" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.e Other Transportation")</f>
-        <v>1.A.3.e Other Transportation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.3.e  Other Transportation")</f>
+        <v>1.A.3.e  Other Transportation</v>
       </c>
       <c r="E16" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13279,8 +13285,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D22" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.1 Solid Fuels")</f>
-        <v>1.B.1 Solid Fuels</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.1  Solid Fuels")</f>
+        <v>1.B.1  Solid Fuels</v>
       </c>
       <c r="E22" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13323,8 +13329,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D24" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.v Distribution of Oil Products")</f>
-        <v>1.B.2.a.v Distribution of Oil Products</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.v  Distribution of Oil Products")</f>
+        <v>1.B.2.a.v  Distribution of Oil Products</v>
       </c>
       <c r="E24" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13345,8 +13351,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D25" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi Other")</f>
-        <v>1.B.2.a.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.a.vi  Other")</f>
+        <v>1.B.2.a.vi  Other</v>
       </c>
       <c r="E25" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13367,8 +13373,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D26" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.v Distribution")</f>
-        <v>1.B.2.b.v Distribution</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.v  Distribution")</f>
+        <v>1.B.2.b.v  Distribution</v>
       </c>
       <c r="E26" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13389,8 +13395,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D27" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi Other")</f>
-        <v>1.B.2.b.vi Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.B.2.b.vi  Other")</f>
+        <v>1.B.2.b.vi  Other</v>
       </c>
       <c r="E27" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13485,8 +13491,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D33" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b Non-Ferrous Metals")</f>
-        <v>1.A.2.b Non-Ferrous Metals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.b  Non-Ferrous Metals")</f>
+        <v>1.A.2.b  Non-Ferrous Metals</v>
       </c>
       <c r="E33" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13507,8 +13513,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D34" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c Chemicals")</f>
-        <v>1.A.2.c Chemicals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.c  Chemicals")</f>
+        <v>1.A.2.c  Chemicals</v>
       </c>
       <c r="E34" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13529,8 +13535,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D35" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d Pulp, Paper and Print")</f>
-        <v>1.A.2.d Pulp, Paper and Print</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.d  Pulp, Paper and Print")</f>
+        <v>1.A.2.d  Pulp, Paper and Print</v>
       </c>
       <c r="E35" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13551,8 +13557,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D36" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.e Food Processing, Beverages and Tobacco")</f>
-        <v>1.A.2.e Food Processing, Beverages and Tobacco</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.e  Food Processing, Beverages and Tobacco")</f>
+        <v>1.A.2.e  Food Processing, Beverages and Tobacco</v>
       </c>
       <c r="E36" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13573,8 +13579,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D37" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.f Non-metallic Minerals")</f>
-        <v>1.A.2.f Non-metallic Minerals</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.f  Non-metallic Minerals")</f>
+        <v>1.A.2.f  Non-metallic Minerals</v>
       </c>
       <c r="E37" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -13595,8 +13601,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D38" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.g Other")</f>
-        <v>1.A.2.g Other</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"1.A.2.g  Other")</f>
+        <v>1.A.2.g  Other</v>
       </c>
       <c r="E38" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14070,8 +14076,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D60" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.B Manure Management")</f>
-        <v>3.B Manure Management</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.B  Manure Management")</f>
+        <v>3.B  Manure Management</v>
       </c>
       <c r="E60" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14092,8 +14098,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D61" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C Rice Cultivation")</f>
-        <v>3.C Rice Cultivation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C  Rice Cultivation")</f>
+        <v>3.C  Rice Cultivation</v>
       </c>
       <c r="E61" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14136,8 +14142,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D63" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A Enteric Fermentation")</f>
-        <v>3.A Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A  Enteric Fermentation")</f>
+        <v>3.A  Enteric Fermentation</v>
       </c>
       <c r="E63" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14158,8 +14164,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D64" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C Rice Cultivation")</f>
-        <v>3.C Rice Cultivation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.C  Rice Cultivation")</f>
+        <v>3.C  Rice Cultivation</v>
       </c>
       <c r="E64" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14202,8 +14208,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D66" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A Enteric Fermentation")</f>
-        <v>3.A Enteric Fermentation</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.A  Enteric Fermentation")</f>
+        <v>3.A  Enteric Fermentation</v>
       </c>
       <c r="E66" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>
@@ -14224,8 +14230,8 @@
         <v>unfccc_annex_1</v>
       </c>
       <c r="D67" s="9" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.B Manure Management")</f>
-        <v>3.B Manure Management</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"3.B  Manure Management")</f>
+        <v>3.B  Manure Management</v>
       </c>
       <c r="E67" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-1.0)</f>

</xml_diff>